<commit_message>
Relative links at possible
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,11 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>Modern Atrium Walkway</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Warm Limewash Studio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added laptop Wise Variabled-PATHS, looping and auto injnectng prompt by pyauto-click
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -1,67 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work-mom\Code-Tools\Full-LC-AUTO\image_prompter\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F77F306A-9D3B-42B4-B5CF-6CEE9EDF9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>KIND</t>
-  </si>
-  <si>
-    <t>USED PHRASE_1</t>
-  </si>
-  <si>
-    <t>BEIGE</t>
-  </si>
-  <si>
-    <t>ICE</t>
-  </si>
-  <si>
-    <t>BLACK-BAGGY</t>
-  </si>
-  <si>
-    <t>Shorts</t>
-  </si>
-  <si>
-    <t>Terracota Style With Plant and Gym equipment in background</t>
-  </si>
-  <si>
-    <t>Pajama</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -80,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -360,44 +385,89 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>KIND</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>USED PHRASE_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BEIGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BLACK-BAGGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Shorts</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Terracota Style With Plant and Gym equipment in background</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Warm Limewash Studio</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pearl Microcement Studio</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Champagne Clay Studio</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Soft Quartz Studio</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Bleached Oak Panel Studio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pajama</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bot-page-scanning for better way to setup tasks in a page
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:AC6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,136 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>Warm Limewash Studio</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pearl Microcement Studio</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Soft Quartz Studio</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bleached Oak Panel Studio</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ivory Fabric Wall Studio</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Cashmere Gradient Studio</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Matte Travertine Studio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Alabaster Arch Studio</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satin Ivory Curve Studio</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Mist Gray Ribbed Studio</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Warm Marble Vein Studio</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Parchment Plaster Studio</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Soft Pebble Panel Studio</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Champagne Suede Studio</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Ivory Fluted Panel Studio</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Bone Grid Panel Studio</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Porcelain Block Studio</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Soft Canvas Panel Studio</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Soft Linen Panel Studio</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Warm Sandstone Slab Studio</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Dove Shadow Panel Studio</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Frosted Resin Studio</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Warm Cork Panel Studio</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Brushed Clay Panel Studio</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Mushroom Felt Studio</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Oyster Composite Studio</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Chalk Mineral Studio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
debug point - image
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/Full-LC-AUTO/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -440,6 +440,11 @@
           <t>Terracota Style With Plant and Gym equipment in background</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Chalk Mineral Studio</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>